<commit_message>
Finish assign to truck (Insertion version))
successfully develop new assign to truck with insertion method get new all time low fitness score(best)
</commit_message>
<xml_diff>
--- a/truck_schedule_output.xlsx
+++ b/truck_schedule_output.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\GitHub\GeneticAlgorithmTruckLife\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D23381-5BBE-4AA1-9BCB-9C0B2E6BD345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="20240201" sheetId="1" r:id="rId1"/>
@@ -24,7 +30,7 @@
     <sheet name="20240215" sheetId="15" r:id="rId15"/>
     <sheet name="20240216" sheetId="16" r:id="rId16"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -736,8 +742,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -800,13 +806,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -844,7 +858,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -878,6 +892,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -912,9 +927,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1087,11 +1103,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1108,17 +1124,17 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>7</v>
       </c>
@@ -1129,11 +1145,11 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1150,7 +1166,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>160</v>
       </c>
@@ -1167,7 +1183,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>161</v>
       </c>
@@ -1181,7 +1197,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>162</v>
       </c>
@@ -1195,7 +1211,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>163</v>
       </c>
@@ -1206,7 +1222,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>164</v>
       </c>
@@ -1217,12 +1233,12 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>171</v>
       </c>
@@ -1233,11 +1249,11 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1254,7 +1270,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>180</v>
       </c>
@@ -1268,7 +1284,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>181</v>
       </c>
@@ -1282,7 +1298,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>182</v>
       </c>
@@ -1296,7 +1312,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>183</v>
       </c>
@@ -1307,7 +1323,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>184</v>
       </c>
@@ -1318,12 +1334,12 @@
         <v>196</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>191</v>
       </c>
@@ -1334,11 +1350,11 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1355,7 +1371,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>200</v>
       </c>
@@ -1369,7 +1385,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>201</v>
       </c>
@@ -1383,7 +1399,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>202</v>
       </c>
@@ -1397,7 +1413,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>203</v>
       </c>
@@ -1411,7 +1427,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>63</v>
       </c>
@@ -1425,12 +1441,12 @@
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>164</v>
       </c>
@@ -1441,11 +1457,11 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1462,7 +1478,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>220</v>
       </c>
@@ -1473,7 +1489,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>221</v>
       </c>
@@ -1484,7 +1500,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>222</v>
       </c>
@@ -1495,12 +1511,12 @@
         <v>230</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>227</v>
       </c>
@@ -1511,20 +1527,20 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1541,17 +1557,17 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
         <v>233</v>
       </c>
@@ -1562,20 +1578,20 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1592,7 +1608,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -1603,7 +1619,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>9</v>
       </c>
@@ -1614,7 +1630,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>10</v>
       </c>
@@ -1631,11 +1647,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1652,7 +1668,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>17</v>
       </c>
@@ -1660,7 +1676,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>18</v>
       </c>
@@ -1668,7 +1684,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>19</v>
       </c>
@@ -1676,7 +1692,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>20</v>
       </c>
@@ -1684,7 +1700,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>21</v>
       </c>
@@ -1698,11 +1714,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1719,7 +1735,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1733,7 +1749,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -1747,7 +1763,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1761,7 +1777,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -1775,7 +1791,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -1789,12 +1805,12 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
         <v>48</v>
       </c>
@@ -1805,11 +1821,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1826,7 +1842,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>49</v>
       </c>
@@ -1837,7 +1853,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -1848,7 +1864,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -1859,7 +1875,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>52</v>
       </c>
@@ -1867,7 +1883,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -1875,12 +1891,12 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>60</v>
       </c>
@@ -1891,11 +1907,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1912,7 +1928,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>64</v>
       </c>
@@ -1929,7 +1945,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>65</v>
       </c>
@@ -1946,7 +1962,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>66</v>
       </c>
@@ -1960,7 +1976,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>67</v>
       </c>
@@ -1974,7 +1990,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>68</v>
       </c>
@@ -1988,7 +2004,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>74</v>
       </c>
@@ -1996,7 +2012,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>75</v>
       </c>
@@ -2010,11 +2026,11 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2031,7 +2047,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>90</v>
       </c>
@@ -2048,7 +2064,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>91</v>
       </c>
@@ -2065,7 +2081,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>92</v>
       </c>
@@ -2082,7 +2098,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>93</v>
       </c>
@@ -2096,7 +2112,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>94</v>
       </c>
@@ -2107,12 +2123,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>106</v>
       </c>
@@ -2123,11 +2139,15 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="4" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2144,7 +2164,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>114</v>
       </c>
@@ -2161,7 +2181,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>115</v>
       </c>
@@ -2178,7 +2198,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>116</v>
       </c>
@@ -2195,7 +2215,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>117</v>
       </c>
@@ -2209,7 +2229,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>118</v>
       </c>
@@ -2220,7 +2240,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>119</v>
       </c>
@@ -2228,7 +2248,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>120</v>
       </c>
@@ -2242,11 +2262,15 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="4" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2263,7 +2287,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>140</v>
       </c>
@@ -2277,7 +2301,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>141</v>
       </c>
@@ -2291,7 +2315,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>142</v>
       </c>
@@ -2305,7 +2329,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>143</v>
       </c>
@@ -2319,7 +2343,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>144</v>
       </c>

</xml_diff>